<commit_message>
fix: calibrate confidence levels in prompt
Initial run returned High on all 23 rows; broadened Medium trigger to
fire on any former target-sector use, retained fit-out/consent, or
'suitable for'/'marketed at' language of any kind — not just
target-sector-specific. Result: 23/23 categories correct, 21/23
confidence correct; 2 false Mediums remain (land plot and former cafe
over-flagged for human review) — accepted as the safer failure mode
over under-flagging
</commit_message>
<xml_diff>
--- a/results/predictions.xlsx
+++ b/results/predictions.xlsx
@@ -471,14 +471,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The listing states it is a former Co-op convenience store, vacant since relocation and offered with vacant possession. Per rules, “former” and “vacant possession” indicate it is not currently operating as a food store or any other category.</t>
+          <t>Listing states a former Co-op convenience store and vacant possession; current use is not operating. Terms like “former” and “vacant” trigger None under the rules, despite prior food retail fit-out and use.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -486,8 +486,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F2" s="2" t="b">
-        <v>0</v>
+      <c r="F2" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -501,14 +501,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Listing is for a plot of land/ancient woodland with potential for development subject to planning. No current operation as a nursery, SEN school, or food store is stated.</t>
+          <t>Current use is a plot of ancient woodland/land; no operating business and no connection to nursery, SEN school, or food retail. Phrases like “opportunity to build” indicate uncommitted use, triggering Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -516,8 +516,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F3" s="1" t="b">
-        <v>0</v>
+      <c r="F3" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -538,7 +538,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Currently fully let as general retail (ground/first floors) with a dance studio (second floor). No indication of a children’s nursery, SEN school, or a food retail store operating on site.</t>
+          <t>Currently fully let as a general retail premises with ancillary storage and a dance studio; no indication of a children’s nursery, SEN school, or food retail tenant. No “former”/vacant language. Therefore not in target sectors.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -561,14 +561,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Listing states it is a former café, the business has ceased trading, and the property is offered with vacant possession. Therefore it is not currently operating as a nursery, SEN school, or food store.</t>
+          <t>Listing states a former café that has ceased trading and is offered with vacant possession. No current nursery, SEN school, or food store operation. Presence of “suitable for”/future-use language warrants Medium confidence per rules.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -576,8 +576,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F5" s="1" t="b">
-        <v>0</v>
+      <c r="F5" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -591,14 +591,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Listing states it is a former doctor’s surgery and markets it as suitable for alternative uses; no current operation as nursery, SEN school, or food store. The term “former” triggers None per rules.</t>
+          <t>Described as a former doctor’s surgery with “ideal for” alternative uses; no current nursery, SEN school, or food store operation stated. Language indicates vacancy/uncommitted use.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -606,8 +606,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F6" s="2" t="b">
-        <v>0</v>
+      <c r="F6" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -628,7 +628,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>The property’s current ground-floor use is a sunbed/tanning shop with a flat above, which is not a nursery, SEN school, or food store. The mention of a nearby Budgens/Premier store is location context and not the subject property.</t>
+          <t>Currently a ground-floor sunbed/tanning shop with a residential flat above. No nursery, SEN school, or food store operation. Nearby convenience store is only a location reference and not the subject property.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Currently operating as a retail shop manufacturing and selling bath products; not a food store, nursery, or SEN school. Current use stated explicitly.</t>
+          <t>Currently a mixed-use property with a retail shop/workshop selling bath products and a holiday apartment. Not a food retail store and not operating as a nursery or SEN school.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The listing is for a public house/freehouse (pub) currently in use as a licensed premises. This is not a nursery, SEN school, or food store, and there are no signals like “former” or “vacant possession” that would change current use.</t>
+          <t>The listing is for a public house/freehouse (pub) currently trading; this is unrelated to nurseries, SEN schools, or food retail. Nearby schools are location context only.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The listing is for a fully let multi-let industrial/trade park. Current use is industrial/trade units, not a nursery, SEN school, or a food retail store. Nearby occupiers mentioned are for location context only.</t>
+          <t>Current use is a fully let industrial/trade park with multiple industrial and trade counter units. No units operate as a nursery, SEN school, or a food retail store; occupiers listed are industrial/logistics (e.g., Royal Mail, DPD, De La Rue).</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Listing describes a fire door manufacturer/joinery business operating from an industrial property, not a nursery, SEN school, or food store.</t>
+          <t>Currently operates as an industrial fire door manufacturer/joinery business; not a nursery, SEN school, or food store.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The asset for sale is a freehold with a long leasehold garage/workshop currently let; the ground-floor retail shop is sold off on a long lease. No current operation as a nursery, SEN school, or food store is stated. Nearby food retailers are only location context. Therefore none of the target sectors apply.</t>
+          <t>Current uses are a garage/workshop (let) and a ground-floor retail shop sold off on a long lease, plus flats. No mention of a nursery, SEN school, or a food retail tenant. Nearby Tesco Express is only a location reference. Development/airspace potential is irrelevant to current use.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -801,14 +801,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The unit is a “blank canvas” marketed to healthcare/medical professionals with refurbishments completing by Aug 2026 and no named current tenant. Language is “suitable for”/versatile space, indicating no current operation. Nearby/adjacent Co-op and other park tenants are not this unit. Therefore it is not currently a nursery, SEN school, or food store.</t>
+          <t>Marketed as a blank-canvas healthcare/medical premises with no named current tenant and no active nursery, SEN school, or food store use. Language like “opportunity for Healthcare and Medical Professionals” and versatile space indicates uncommitted current use; adjacency to Co-Op is just location.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -816,8 +816,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F13" s="2" t="b">
-        <v>0</v>
+      <c r="F13" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -838,7 +838,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>The listing explicitly states it is currently let to and operated by an independent special educational needs provider and is "currently operating as independent SEN school," with an active lease (c. 11 years unexpired). The mention of "former grammar school" refers to historic use, not current use.</t>
+          <t>Explicitly stated as currently let to and operated by an independent special educational needs provider; listing says ‘Currently operating as independent SEN school’ with 11 years unexpired on the lease. ‘Former grammar school’ refers to historic use, not current.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Currently let to a vape/e-cigarette retailer and a hairdressing salon, with residential flats above. No childcare, SEN education, or food retail operation, and the listing explicitly notes no consent for those uses.</t>
+          <t>Currently let to a vape/e-cigarette retailer and a hairdressing salon with no consent for childcare, education, or food retail. These uses are unrelated to nursery, SEN school, or food store.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -891,14 +891,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Currently operating as a car showroom with attached residence; mentions of being ideal for other uses are speculative. Not a nursery, SEN school, or food store.</t>
+          <t>Currently a car showroom with residence; no nursery, SEN school, or food retail operation. Mentions “suitable for” other uses but no named current tenant in target sectors, so classify as None and flag Medium due to the ‘suitable for’ language.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -906,8 +906,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F16" s="2" t="b">
-        <v>0</v>
+      <c r="F16" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -928,7 +928,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>The listing explicitly describes an established, currently operating children’s day nursery (registered for 75, Good Ofsted, open year-round, currently at ~50% occupancy). No “former” or vacancy language present.</t>
+          <t>Listing explicitly describes an established, currently operating children’s day nursery (registered for 75, Good Ofsted, open year-round, staffed and trading).</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -951,14 +951,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Listing states “Vacant FREEHOLD Nursery Building” and “offered with full vacant possession.” Per rule 2, these phrases signal None, regardless of nursery configuration or past operation.</t>
+          <t>Listing states “Vacant FREEHOLD Nursery Building” and “will be offered with full vacant possession,” which per Rule 2 signals None, despite mentioning it is currently configured/operated as a nursery. Strong nursery connection but being sold vacant merits Medium confidence.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -966,8 +966,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F18" s="2" t="b">
-        <v>0</v>
+      <c r="F18" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -981,14 +981,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>This is an airspace development opportunity to build apartments; per rule 5 we classify what is being sold (airspace), not the underlying tenant. Although the ground floor is let to Sainsbury’s, the listing is for the rooftop development rights, not a currently operating food store.</t>
+          <t>This is a sale of airspace development rights to create apartments. Although the ground floor is let to Sainsbury’s (a food store), Rule 5 says classify what is being sold—the airspace—so it is not a current target-sector use. Confidence is Medium because it involves airspace above a target-sector tenant.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -996,8 +996,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F19" s="2" t="b">
-        <v>0</v>
+      <c r="F19" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Industrial/warehouse complex marketed for manufacturing/storage uses; no indication of current operation as nursery, SEN school, or food store. Language like “suitable for” confirms not currently in those sectors.</t>
+          <t>Industrial/warehouse complex with uses for manufacturing, storage, engineering, and distribution. No current operation as a nursery, SEN school, or food retail store; clearly unrelated to target sectors.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1041,14 +1041,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The listing states the property is offered with full vacant possession and is a vacant freehold nursery building. Despite nursery fit-out, it is not currently operating. Per Rule 2, “vacant possession” signals None.</t>
+          <t>Listing states “Vacant FREEHOLD Nursery Building” and “offered…with full vacant possession,” so it is not currently operating. Despite nursery fit-out and sector language, current use is vacant per Rule 2.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1056,8 +1056,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F21" s="2" t="b">
-        <v>0</v>
+      <c r="F21" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Listing explicitly states the unit is used as a small convenience store and is let on a current lease with the business remaining unaffected, confirming current food retail operation.</t>
+          <t>Listing states the unit is currently used as a small convenience store and is let on a 9-year FRI lease with the business remaining unaffected by the sale, confirming active food retail use.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1101,14 +1101,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>The listing states the unit is vacant and ‘most recently trading as’ a nursery with the operator’s ‘lease expired’. These phrases explicitly indicate it is not currently operating. Despite D1 consent and nursery fit-out, this is marketing/suitability, not current use.</t>
+          <t>Listing states the unit is vacant and ‘most recently trading as’ a nursery with the operator’s ‘lease expired’—phrases that signal None under the rules. D1 nursery consent and retained nursery fit-out indicate former/suitable use, not current operation.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1116,8 +1116,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F23" s="2" t="b">
-        <v>0</v>
+      <c r="F23" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1131,14 +1131,14 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>The listing repeatedly states it is a former Costcutter supermarket and will be sold vacant. Per rules, terms like “former” and “vacant” mean it is not currently operating as a food store or other target use.</t>
+          <t>Described repeatedly as a former Costcutter supermarket, sold vacant with no lease/third-party agreements and “suitable for alternative uses.” Current use is not an operating food store.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1146,8 +1146,8 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F24" s="2" t="b">
-        <v>0</v>
+      <c r="F24" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>